<commit_message>
feat: routes + controller
</commit_message>
<xml_diff>
--- a/Doc Backend/Journal-de-Travail_ReynaudThomas-Backend.xlsx
+++ b/Doc Backend/Journal-de-Travail_ReynaudThomas-Backend.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk84vtk\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk84vtk\Documents\GitHub\Passion-Lecture\Doc Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDA1B9E0-4CDB-423B-9685-CB109F0A1F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F1C9C5-62EF-4A12-B5C8-6215DACB8AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="29505" yWindow="1335" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="39">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -143,6 +143,21 @@
   </si>
   <si>
     <t>J'ai aidé ryan avec le MCD MLD pour que tt soit en ordre avant de le faire verifier au prof</t>
+  </si>
+  <si>
+    <t>J'ai recupérer mes exercices et j'ai relu la doc des validators ainsi que mes exercices pour commencer les controllers. Je vais commencer par le controller books.</t>
+  </si>
+  <si>
+    <t>J'ai regarder les models et les migrations avec ryan</t>
+  </si>
+  <si>
+    <t>J'ai commencé a faire les controllers (en premier le booksController)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J'ai terminé le controller books ainsi que son validator </t>
+  </si>
+  <si>
+    <t>Problème de version avec github etc on a du refaire certaines parties et corriger certaines choses.</t>
   </si>
 </sst>
 </file>
@@ -1150,16 +1165,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>30</c:v>
+                  <c:v>115</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>105</c:v>
+                  <c:v>240</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>90</c:v>
+                  <c:v>170</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2005,16 +2020,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.13333333333333333</c:v>
+                  <c:v>0.21904761904761905</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.46666666666666667</c:v>
+                  <c:v>0.45714285714285713</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.4</c:v>
+                  <c:v>0.32380952380952382</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4249,7 +4264,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>3 heures 45 minutes</v>
+        <v>8 heures 45 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4262,15 +4277,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>105</v>
+        <v>225</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>225</v>
+        <v>525</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4382,16 +4397,26 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="62" t="str">
+    <row r="10" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="62">
         <f>IF(ISBLANK(B10),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B10))</f>
-        <v/>
-      </c>
-      <c r="B10" s="30"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="23"/>
+        <v>19</v>
+      </c>
+      <c r="B10" s="30">
+        <v>46146</v>
+      </c>
+      <c r="C10" s="31">
+        <v>1</v>
+      </c>
+      <c r="D10" s="32">
+        <v>20</v>
+      </c>
+      <c r="E10" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>34</v>
+      </c>
       <c r="G10" s="39"/>
       <c r="M10" t="s">
         <v>15</v>
@@ -4410,9 +4435,15 @@
       </c>
       <c r="B11" s="34"/>
       <c r="C11" s="35"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="23"/>
+      <c r="D11" s="36">
+        <v>40</v>
+      </c>
+      <c r="E11" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>35</v>
+      </c>
       <c r="G11" s="40"/>
       <c r="M11" t="s">
         <v>16</v>
@@ -4431,9 +4462,15 @@
       </c>
       <c r="B12" s="30"/>
       <c r="C12" s="31"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="23"/>
+      <c r="D12" s="32">
+        <v>15</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>36</v>
+      </c>
       <c r="G12" s="39"/>
       <c r="M12" t="s">
         <v>17</v>
@@ -4446,15 +4483,23 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="63" t="str">
+      <c r="A13" s="63">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
-        <v/>
-      </c>
-      <c r="B13" s="34"/>
-      <c r="C13" s="35"/>
+        <v>14</v>
+      </c>
+      <c r="B13" s="34">
+        <v>46117</v>
+      </c>
+      <c r="C13" s="35">
+        <v>2</v>
+      </c>
       <c r="D13" s="36"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="23"/>
+      <c r="E13" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>37</v>
+      </c>
       <c r="G13" s="40"/>
       <c r="N13">
         <v>6</v>
@@ -4470,9 +4515,15 @@
       </c>
       <c r="B14" s="30"/>
       <c r="C14" s="31"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="23"/>
+      <c r="D14" s="32">
+        <v>45</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>38</v>
+      </c>
       <c r="G14" s="39"/>
       <c r="N14">
         <v>7</v>
@@ -10853,11 +10904,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>30</v>
+        <v>115</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>30</v>
+        <v>115</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10865,11 +10916,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>0 h 30 min</v>
+        <v>1 h 55 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.13333333333333333</v>
+        <v>0.21904761904761905</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10886,15 +10937,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>105</v>
+        <v>240</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10902,11 +10953,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>1 h 45 min</v>
+        <v>4 h 00 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.46666666666666667</v>
+        <v>0.45714285714285713</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10960,15 +11011,15 @@
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>90</v>
+        <v>170</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -10976,11 +11027,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>1 h 30 min</v>
+        <v>2 h 50 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.4</v>
+        <v>0.32380952380952382</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11032,26 +11083,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>105</v>
+        <v>225</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>225</v>
+        <v>525</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>3 h 45 min</v>
+        <v>8 h 45 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>4.1666666666666664E-2</v>
+        <v>9.7222222222222224E-2</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>28</v>
@@ -11090,17 +11141,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="5bf905bc6027d3a3176cf398b6d748a7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cdc8923a5f0a5cb2ad217e59a32ed26c" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11289,6 +11329,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11299,17 +11350,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB23EBB1-226D-48F9-BD4F-72DBF2899D35}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11328,6 +11368,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
fix: typo of autor to author
</commit_message>
<xml_diff>
--- a/Doc Backend/Journal-de-Travail_ReynaudThomas-Backend.xlsx
+++ b/Doc Backend/Journal-de-Travail_ReynaudThomas-Backend.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk84vtk\Documents\GitHub\Passion-Lecture\Doc Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0F1C9C5-62EF-4A12-B5C8-6215DACB8AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{279EEA8B-83FE-4AF9-A760-28582AB7B107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29505" yWindow="1335" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="5490" yWindow="945" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="42">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -158,6 +158,15 @@
   </si>
   <si>
     <t>Problème de version avec github etc on a du refaire certaines parties et corriger certaines choses.</t>
+  </si>
+  <si>
+    <t>J'ai reprise mon controller books car certaines fonctionnalitées manquaient</t>
+  </si>
+  <si>
+    <t>J'ai fais les tests api avec bruno notemment authors ils marchent tous</t>
+  </si>
+  <si>
+    <t>J'ai aussi commencé les tests apis books quelqu'uns ne marchent pas je dois commencé l'auth</t>
   </si>
 </sst>
 </file>
@@ -1168,10 +1177,10 @@
                   <c:v>115</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>240</c:v>
+                  <c:v>300</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>135</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>170</c:v>
@@ -2020,16 +2029,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.21904761904761905</c:v>
+                  <c:v>0.15972222222222221</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.45714285714285713</c:v>
+                  <c:v>0.41666666666666669</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>0.1875</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.32380952380952382</c:v>
+                  <c:v>0.2361111111111111</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4264,7 +4273,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>8 heures 45 minutes</v>
+        <v>12 heures 0 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4277,15 +4286,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>300</v>
+        <v>420</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>225</v>
+        <v>300</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>525</v>
+        <v>720</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4485,10 +4494,10 @@
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="63">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B13" s="34">
-        <v>46117</v>
+        <v>46147</v>
       </c>
       <c r="C13" s="35">
         <v>2</v>
@@ -4538,10 +4547,16 @@
         <v/>
       </c>
       <c r="B15" s="34"/>
-      <c r="C15" s="35"/>
+      <c r="C15" s="35">
+        <v>1</v>
+      </c>
       <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="23"/>
+      <c r="E15" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>39</v>
+      </c>
       <c r="G15" s="40"/>
       <c r="N15">
         <v>8</v>
@@ -4551,15 +4566,25 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="62" t="str">
+      <c r="A16" s="62">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
-        <v/>
-      </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="23"/>
+        <v>20</v>
+      </c>
+      <c r="B16" s="30">
+        <v>46153</v>
+      </c>
+      <c r="C16" s="31">
+        <v>1</v>
+      </c>
+      <c r="D16" s="32">
+        <v>20</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>40</v>
+      </c>
       <c r="G16" s="39"/>
       <c r="O16">
         <v>40</v>
@@ -4572,20 +4597,28 @@
       </c>
       <c r="B17" s="34"/>
       <c r="C17" s="35"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="23"/>
+      <c r="D17" s="36">
+        <v>55</v>
+      </c>
+      <c r="E17" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>41</v>
+      </c>
       <c r="G17" s="40"/>
       <c r="O17">
         <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="62" t="str">
+      <c r="A18" s="62">
         <f>IF(ISBLANK(B18),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B18))</f>
-        <v/>
-      </c>
-      <c r="B18" s="30"/>
+        <v>20</v>
+      </c>
+      <c r="B18" s="30">
+        <v>46154</v>
+      </c>
       <c r="C18" s="31"/>
       <c r="D18" s="32"/>
       <c r="E18" s="33"/>
@@ -10920,7 +10953,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.21904761904761905</v>
+        <v>0.15972222222222221</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10937,7 +10970,7 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
@@ -10945,7 +10978,7 @@
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10953,11 +10986,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>4 h 00 min</v>
+        <v>5 h 00 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.45714285714285713</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10974,15 +11007,15 @@
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E8,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B8">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E8,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="C8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="E8" s="76" t="str">
         <f>'Journal de travail'!M10</f>
@@ -10990,11 +11023,11 @@
       </c>
       <c r="F8" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 00 min</v>
+        <v>2 h 15 min</v>
       </c>
       <c r="G8" s="72">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.1875</v>
       </c>
       <c r="L8" s="54" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11031,7 +11064,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.32380952380952382</v>
+        <v>0.2361111111111111</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11083,26 +11116,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>300</v>
+        <v>420</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>225</v>
+        <v>300</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>525</v>
+        <v>720</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>8 h 45 min</v>
+        <v>12 h 00 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>9.7222222222222224E-2</v>
+        <v>0.13333333333333333</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>28</v>
@@ -11141,6 +11174,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="5bf905bc6027d3a3176cf398b6d748a7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cdc8923a5f0a5cb2ad217e59a32ed26c" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11329,17 +11373,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11350,6 +11383,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB23EBB1-226D-48F9-BD4F-72DBF2899D35}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11368,17 +11412,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
doc: fichier .txt verbes HTTP + jdt
</commit_message>
<xml_diff>
--- a/Doc Backend/Journal-de-Travail_ReynaudThomas-Backend.xlsx
+++ b/Doc Backend/Journal-de-Travail_ReynaudThomas-Backend.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk84vtk\Documents\GitHub\Passion-Lecture\Doc Backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{279EEA8B-83FE-4AF9-A760-28582AB7B107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3326EA0D-7F61-4504-8A23-EC8E252ABD42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5490" yWindow="945" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="46">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -167,6 +167,18 @@
   </si>
   <si>
     <t>J'ai aussi commencé les tests apis books quelqu'uns ne marchent pas je dois commencé l'auth</t>
+  </si>
+  <si>
+    <t>J'ai changé la typo de autor to authors pour des raisons de simplifications</t>
+  </si>
+  <si>
+    <t>J'ai fais le controller auth avec login et register et je les aient liés avec books pour que l'on ne puisse pas créer de livre sans être connecté</t>
+  </si>
+  <si>
+    <t>J'ai fais les tests api de tous les controllers avec le runner, et avec ryan nous avons eu des problèmes d'ordre mais finalement tout les test passent + nous avons fais l'évaluation des 80% et nous sommes dans les temps</t>
+  </si>
+  <si>
+    <t>J'ai fais le fichier txt des verbes HTTP</t>
   </si>
 </sst>
 </file>
@@ -1174,16 +1186,16 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>115</c:v>
+                  <c:v>160</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>300</c:v>
+                  <c:v>390</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>135</c:v>
+                  <c:v>180</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>170</c:v>
+                  <c:v>215</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2029,16 +2041,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.15972222222222221</c:v>
+                  <c:v>0.1693121693121693</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.41666666666666669</c:v>
+                  <c:v>0.41269841269841268</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1875</c:v>
+                  <c:v>0.19047619047619047</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.2361111111111111</c:v>
+                  <c:v>0.2275132275132275</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4273,7 +4285,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>12 heures 0 minutes</v>
+        <v>15 heures 45 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4286,15 +4298,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>300</v>
+        <v>465</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>720</v>
+        <v>945</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4620,39 +4632,59 @@
         <v>46154</v>
       </c>
       <c r="C18" s="31"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="23"/>
+      <c r="D18" s="32">
+        <v>45</v>
+      </c>
+      <c r="E18" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>42</v>
+      </c>
       <c r="G18" s="39"/>
       <c r="O18">
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A19" s="63" t="str">
         <f>IF(ISBLANK(B19),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B19))</f>
         <v/>
       </c>
       <c r="B19" s="34"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="23"/>
+      <c r="C19" s="35">
+        <v>1</v>
+      </c>
+      <c r="D19" s="36">
+        <v>30</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>43</v>
+      </c>
       <c r="G19" s="40"/>
       <c r="O19">
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A20" s="62" t="str">
         <f>IF(ISBLANK(B20),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B20))</f>
         <v/>
       </c>
       <c r="B20" s="30"/>
       <c r="C20" s="31"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="23"/>
+      <c r="D20" s="32">
+        <v>45</v>
+      </c>
+      <c r="E20" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>44</v>
+      </c>
       <c r="G20" s="39"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -4662,9 +4694,15 @@
       </c>
       <c r="B21" s="34"/>
       <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="23"/>
+      <c r="D21" s="36">
+        <v>45</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>45</v>
+      </c>
       <c r="G21" s="40"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -10937,11 +10975,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10949,11 +10987,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>1 h 55 min</v>
+        <v>2 h 40 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.15972222222222221</v>
+        <v>0.1693121693121693</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10970,15 +11008,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>300</v>
+        <v>390</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10986,11 +11024,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>5 h 00 min</v>
+        <v>6 h 30 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.41666666666666669</v>
+        <v>0.41269841269841268</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11011,11 +11049,11 @@
       </c>
       <c r="B8">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E8,'Journal de travail'!$D$7:$D$532)</f>
-        <v>75</v>
+        <v>120</v>
       </c>
       <c r="C8">
         <f t="shared" si="0"/>
-        <v>135</v>
+        <v>180</v>
       </c>
       <c r="E8" s="76" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11023,11 +11061,11 @@
       </c>
       <c r="F8" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>2 h 15 min</v>
+        <v>3 h 00 min</v>
       </c>
       <c r="G8" s="72">
         <f t="shared" si="2"/>
-        <v>0.1875</v>
+        <v>0.19047619047619047</v>
       </c>
       <c r="L8" s="54" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11048,11 +11086,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>50</v>
+        <v>95</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>170</v>
+        <v>215</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11060,11 +11098,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>2 h 50 min</v>
+        <v>3 h 35 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.2361111111111111</v>
+        <v>0.2275132275132275</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11116,26 +11154,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>300</v>
+        <v>465</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>720</v>
+        <v>945</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>12 h 00 min</v>
+        <v>15 h 45 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.13333333333333333</v>
+        <v>0.17499999999999999</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>28</v>
@@ -11174,17 +11212,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="5bf905bc6027d3a3176cf398b6d748a7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cdc8923a5f0a5cb2ad217e59a32ed26c" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11373,6 +11400,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11383,17 +11421,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB23EBB1-226D-48F9-BD4F-72DBF2899D35}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11412,6 +11439,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>